<commit_message>
Add channel performance report generation and update js_api integration
</commit_message>
<xml_diff>
--- a/templates/Channel Performance Header example.xlsx
+++ b/templates/Channel Performance Header example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://georgiancollege-my.sharepoint.com/personal/amy_hutchinson_georgiancollege_ca/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/superq/academic/automation-tool/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1169DCC-56F4-490D-805D-81895D9C260B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F6F8C5E-896C-CE47-93A1-737FDC8026DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11235" xr2:uid="{01AB0956-5F3F-42DF-8DDC-FAE904BD88A8}"/>
+    <workbookView xWindow="740" yWindow="740" windowWidth="21600" windowHeight="11240" xr2:uid="{01AB0956-5F3F-42DF-8DDC-FAE904BD88A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Month</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>Blank</t>
+  </si>
+  <si>
+    <t>w</t>
   </si>
 </sst>
 </file>
@@ -506,10 +509,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15853C3E-558A-42AC-8779-CD2F670478FB}">
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:U9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -572,6 +575,11 @@
       </c>
       <c r="U1" s="3" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="F9" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>